<commit_message>
plots and BOM update
</commit_message>
<xml_diff>
--- a/resources/v0.1.2/design_documents/BOM-V0.1.2.xlsx
+++ b/resources/v0.1.2/design_documents/BOM-V0.1.2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c1ed1b07ceb518fe/Documents/GitHub/core2s/resources/v0.1.2/design_documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{55AB40B0-6C17-4ECF-ABEA-EBBE2E37FDFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EEF25476-B12E-45D4-A545-B6A7F31C32AC}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{55AB40B0-6C17-4ECF-ABEA-EBBE2E37FDFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D6A14642-71D4-43AF-B637-B77EDED742B9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="308">
   <si>
     <t>Total Cost</t>
   </si>
@@ -954,6 +954,12 @@
   </si>
   <si>
     <t>MDR-40-48 100-240VAC</t>
+  </si>
+  <si>
+    <t>Flange, 304/304L Stainless Steel, Metal Pipe Flange - 60WJ74|4381000040 - Grainger</t>
+  </si>
+  <si>
+    <t>Flange  Blind ("plug")</t>
   </si>
 </sst>
 </file>
@@ -1370,6 +1376,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3AC99790-742C-414B-AF83-048E0365A8B5}" name="Table1" displayName="Table1" ref="A1:K120" totalsRowShown="0" tableBorderDxfId="7">
   <autoFilter ref="A1:K120" xr:uid="{3AC99790-742C-414B-AF83-048E0365A8B5}"/>
@@ -4615,7 +4625,9 @@
       <c r="H119" s="10"/>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A120" s="29"/>
+      <c r="A120" s="29" t="s">
+        <v>307</v>
+      </c>
       <c r="B120" s="23"/>
       <c r="C120" s="10"/>
       <c r="D120" s="30"/>
@@ -4624,7 +4636,9 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="H120" s="10"/>
+      <c r="H120" s="1" t="s">
+        <v>306</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -4739,11 +4753,12 @@
     <hyperlink ref="H116" r:id="rId108" display="https://www.grainger.com/product/20KF99?RIID=51819294775&amp;GID=729415832&amp;mid=OrderConfirmation_REST&amp;rfe=a98025ace82cfe3e9959eb0e2dd5f9501b4a446af591eb4540e15aea507809d7&amp;gucid=EMT:11126144:Item:CSM-323&amp;emcid=NA:Item" xr:uid="{2C0D4D21-381D-4DE0-8627-C5CDD08AC966}"/>
     <hyperlink ref="H117" r:id="rId109" display="https://www.grainger.com/product/Compression-Lug-3-8-in-Stud-24C366" xr:uid="{969E4A0C-E52F-4A17-A6F5-A3D01F24676B}"/>
     <hyperlink ref="H118" r:id="rId110" display="https://www.digikey.com/en/products/detail/advantech-corporation/bb-mdr-40-48/7426468" xr:uid="{65E538F7-DA33-4388-B23E-404C55813446}"/>
+    <hyperlink ref="H120" r:id="rId111" display="https://www.grainger.com/product/Metal-Pipe-Flange-Flange-60WJ74" xr:uid="{851EBC08-2ED2-4124-B23F-E667A9F9321B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId111"/>
+  <pageSetup orientation="portrait" r:id="rId112"/>
   <tableParts count="1">
-    <tablePart r:id="rId112"/>
+    <tablePart r:id="rId113"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>